<commit_message>
Added three new profiles and added Anand Meherwade's photograph
</commit_message>
<xml_diff>
--- a/files/member_list.xlsx
+++ b/files/member_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanayanair/Documents/Inventree/members/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{D5D7036B-0870-C144-BD35-A3504AE72AFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF7FA09F-EA64-B047-8F8B-AE8F8887635F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="500" windowWidth="28040" windowHeight="16360" xr2:uid="{9635C76B-74B9-1442-AF08-BD1D1FC844B7}"/>
+    <workbookView xWindow="28960" yWindow="660" windowWidth="38080" windowHeight="20780" xr2:uid="{9635C76B-74B9-1442-AF08-BD1D1FC844B7}"/>
   </bookViews>
   <sheets>
     <sheet name="member_list" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="430">
   <si>
     <t>memberID</t>
   </si>
@@ -1289,13 +1289,34 @@
   </si>
   <si>
     <t>Roy</t>
+  </si>
+  <si>
+    <t>M44</t>
+  </si>
+  <si>
+    <t>Kukke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prasanna J. </t>
+  </si>
+  <si>
+    <t>Data scientist</t>
+  </si>
+  <si>
+    <t>Indian Institute of Science</t>
+  </si>
+  <si>
+    <t>kukkeprasannaj@gmail.com</t>
+  </si>
+  <si>
+    <t>differential equations, computational fluid dynamics, forest dynamics, fire ecology</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1442,6 +1463,11 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow (Body)"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1786,10 +1812,11 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="42"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2166,7 +2193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89131DAE-5091-BD4D-8A8C-CC0C00D895DA}">
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
@@ -3922,9 +3949,42 @@
         <v>103</v>
       </c>
     </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>423</v>
+      </c>
+      <c r="B45" t="s">
+        <v>424</v>
+      </c>
+      <c r="C45" t="s">
+        <v>425</v>
+      </c>
+      <c r="D45" t="s">
+        <v>426</v>
+      </c>
+      <c r="E45" t="s">
+        <v>427</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="L45" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="M45" t="s">
+        <v>155</v>
+      </c>
+      <c r="N45" t="s">
+        <v>129</v>
+      </c>
+      <c r="O45" t="s">
+        <v>103</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F44" r:id="rId1" display="mailto:psroy13@gmail.com" xr:uid="{39936BE1-F42F-BC47-B9D2-347C446B0534}"/>
+    <hyperlink ref="F45" r:id="rId2" display="mailto:kukkeprasannaj@gmail.com" xr:uid="{7E8B6291-2D5A-4D43-A88B-553579A75196}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>